<commit_message>
M1: Tách cấu trúc Độc lập Trang chủ Dashboard - Update UI of dashboard_view
</commit_message>
<xml_diff>
--- a/.00_resource/EduStayAI Roadmap.xlsx
+++ b/.00_resource/EduStayAI Roadmap.xlsx
@@ -9,13 +9,14 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7310" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7310"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
     <sheet name="Milestones" sheetId="4" r:id="rId2"/>
-    <sheet name="Notes" sheetId="3" r:id="rId3"/>
-    <sheet name="temp" sheetId="2" r:id="rId4"/>
+    <sheet name="Requirements" sheetId="5" r:id="rId3"/>
+    <sheet name="Notes" sheetId="3" r:id="rId4"/>
+    <sheet name="temp" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="471">
   <si>
     <t>Roadmap Phát Triển Sản Phẩm &amp; Marketing (1 Người + AI)</t>
   </si>
@@ -651,13 +652,840 @@
   </si>
   <si>
     <t>T01-11/2028</t>
+  </si>
+  <si>
+    <t>1. User</t>
+  </si>
+  <si>
+    <t>Ví dụ:</t>
+  </si>
+  <si>
+    <t>Tháng 6/2026 launch app</t>
+  </si>
+  <si>
+    <t>Có 1.000 người đăng ký</t>
+  </si>
+  <si>
+    <t>=&gt; KPI User = 1.000</t>
+  </si>
+  <si>
+    <t>Tuy nhiên chỉ số này dễ "ảo".</t>
+  </si>
+  <si>
+    <t>1.000 người đăng ký</t>
+  </si>
+  <si>
+    <t>Chỉ 10 người còn dùng</t>
+  </si>
+  <si>
+    <t>=&gt; App vẫn thất bại.</t>
+  </si>
+  <si>
+    <t>2. DAU (Daily Active Users)</t>
+  </si>
+  <si>
+    <t>Là số người thực sự sử dụng app mỗi ngày.</t>
+  </si>
+  <si>
+    <t>Ngày</t>
+  </si>
+  <si>
+    <t>User mở app</t>
+  </si>
+  <si>
+    <t>Thứ 2</t>
+  </si>
+  <si>
+    <t>Thứ 3</t>
+  </si>
+  <si>
+    <t>Thứ 4</t>
+  </si>
+  <si>
+    <t>Thứ 5</t>
+  </si>
+  <si>
+    <t>=&gt; DAU trung bình khoảng 110.</t>
+  </si>
+  <si>
+    <t>Đối với app học tập mới:</t>
+  </si>
+  <si>
+    <t>DAU 100 là khá ổn</t>
+  </si>
+  <si>
+    <t>DAU 500 là tốt</t>
+  </si>
+  <si>
+    <t>DAU 1.000+ là rất tốt</t>
+  </si>
+  <si>
+    <t>3. D7 Retention</t>
+  </si>
+  <si>
+    <t>Đây là KPI quan trọng nhất.</t>
+  </si>
+  <si>
+    <t>Cách tính:</t>
+  </si>
+  <si>
+    <t>Ví dụ ngày 1 có:</t>
+  </si>
+  <si>
+    <t>100 người đăng ký</t>
+  </si>
+  <si>
+    <t>Sau 7 ngày:</t>
+  </si>
+  <si>
+    <t>25 người vẫn quay lại học</t>
+  </si>
+  <si>
+    <t>=&gt; D7 = 25%</t>
+  </si>
+  <si>
+    <t>Công thức:</t>
+  </si>
+  <si>
+    <t>D7 Retention=User quay lại ngaˋy thứ 7User đa˘ng kyˊ ban đa^ˋu×100%D7\ Retention = \frac{User\ quay\ lại\ ngày\ thứ\ 7}{User\ đăng\ ký\ ban\ đầu} \times 100\%D7 Retention=User đa˘ng kyˊ​ ban đa^ˋuUser quay lại ngaˋy thứ 7​×100%</t>
+  </si>
+  <si>
+    <t>D7 bao nhiêu là tốt?</t>
+  </si>
+  <si>
+    <t>D7</t>
+  </si>
+  <si>
+    <t>Đánh giá</t>
+  </si>
+  <si>
+    <t>&lt;10%</t>
+  </si>
+  <si>
+    <t>Rất tệ</t>
+  </si>
+  <si>
+    <t>10-20%</t>
+  </si>
+  <si>
+    <t>Trung bình</t>
+  </si>
+  <si>
+    <t>20-30%</t>
+  </si>
+  <si>
+    <t>Tốt</t>
+  </si>
+  <si>
+    <t>30-40%</t>
+  </si>
+  <si>
+    <t>Rất tốt</t>
+  </si>
+  <si>
+    <t>&gt;40%</t>
+  </si>
+  <si>
+    <t>Xuất sắc</t>
+  </si>
+  <si>
+    <t>Đối với app học tiếng Anh mới:</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Mục tiêu ban đầu: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>20%</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Sau khi tối ưu: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>25-30%</t>
+    </r>
+  </si>
+  <si>
+    <t>Ví dụ thực tế cho app của bạn</t>
+  </si>
+  <si>
+    <t>Giả sử sau 3 tháng:</t>
+  </si>
+  <si>
+    <t>DAU = 120</t>
+  </si>
+  <si>
+    <t>D7 = 25%</t>
+  </si>
+  <si>
+    <t>=&gt; Đây là tín hiệu khá tốt.</t>
+  </si>
+  <si>
+    <t>Tiếp tục 6 tháng:</t>
+  </si>
+  <si>
+    <t>5.000 user</t>
+  </si>
+  <si>
+    <t>DAU = 500</t>
+  </si>
+  <si>
+    <t>D7 = 30%</t>
+  </si>
+  <si>
+    <t>=&gt; Lúc này có thể bắt đầu mở Premium.</t>
+  </si>
+  <si>
+    <t>Nếu chỉ được chọn 1 KPI để theo dõi</t>
+  </si>
+  <si>
+    <t>Thì hãy theo:</t>
+  </si>
+  <si>
+    <t>D7 Retention</t>
+  </si>
+  <si>
+    <t>Vì:</t>
+  </si>
+  <si>
+    <t>User có thể mua quảng cáo được.</t>
+  </si>
+  <si>
+    <t>Download có thể mua được.</t>
+  </si>
+  <si>
+    <t>Nhưng nếu người dùng không quay lại học thì app không có giá trị.</t>
+  </si>
+  <si>
+    <t>Đối với app học tiếng Anh của bạn, tôi sẽ ưu tiên KPI theo thứ tự:</t>
+  </si>
+  <si>
+    <r>
+      <t>1. D7 Retention</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (quan trọng nhất)</t>
+    </r>
+  </si>
+  <si>
+    <t>2. DAU</t>
+  </si>
+  <si>
+    <t>3. Số phút học trung bình/ngày</t>
+  </si>
+  <si>
+    <t>4. Tỷ lệ hoàn thành bài học</t>
+  </si>
+  <si>
+    <t>5. Tổng số user đăng ký</t>
+  </si>
+  <si>
+    <t>Đó là bộ KPI mà các app như Duolingo hay ELSA Speak cũng rất quan tâm trong giai đoạn đầu tăng trưởng.</t>
+  </si>
+  <si>
+    <t>Edu-Stay AI - Product Backlog &amp; Roadmap</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Epic</t>
+  </si>
+  <si>
+    <t>Feature / Requirement</t>
+  </si>
+  <si>
+    <t>User Value</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Effort</t>
+  </si>
+  <si>
+    <t>Release</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Dependency</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>UI-001</t>
+  </si>
+  <si>
+    <t>UX/UI</t>
+  </si>
+  <si>
+    <t>Refactor toàn bộ UI theo hướng mobile-first</t>
+  </si>
+  <si>
+    <t>Tăng usability</t>
+  </si>
+  <si>
+    <t>P0</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>MVP</t>
+  </si>
+  <si>
+    <t>Todo</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Mobile là kênh sử dụng chính</t>
+  </si>
+  <si>
+    <t>UI-002</t>
+  </si>
+  <si>
+    <t>Giảm scroll, tối ưu "vùng đất vàng"</t>
+  </si>
+  <si>
+    <t>Tăng engagement</t>
+  </si>
+  <si>
+    <t>Ưu tiên thông tin quan trọng ở first screen</t>
+  </si>
+  <si>
+    <t>UI-003</t>
+  </si>
+  <si>
+    <t>Tách Dashboard và Lesson thành 2 page riêng</t>
+  </si>
+  <si>
+    <t>Điều hướng rõ ràng</t>
+  </si>
+  <si>
+    <t>Navigation đơn giản hơn</t>
+  </si>
+  <si>
+    <t>UI-004</t>
+  </si>
+  <si>
+    <t>Tăng độ tương phản text trên mobile</t>
+  </si>
+  <si>
+    <t>Cải thiện khả năng đọc</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>Fix button, radio, option text</t>
+  </si>
+  <si>
+    <t>UI-005</t>
+  </si>
+  <si>
+    <t>Thu nhỏ logo show, avatar user</t>
+  </si>
+  <si>
+    <t>Tối ưu không gian</t>
+  </si>
+  <si>
+    <t>Giảm kích thước 30-50%</t>
+  </si>
+  <si>
+    <t>UI-006</t>
+  </si>
+  <si>
+    <t>Thiết kế lại left menu</t>
+  </si>
+  <si>
+    <t>Gọn gàng hơn</t>
+  </si>
+  <si>
+    <t>Bỏ thông tin test</t>
+  </si>
+  <si>
+    <t>UI-007</t>
+  </si>
+  <si>
+    <t>Rút gọn wording cho Gen Z</t>
+  </si>
+  <si>
+    <t>Dễ sử dụng</t>
+  </si>
+  <si>
+    <t>Hạn chế text dài</t>
+  </si>
+  <si>
+    <t>UI-008</t>
+  </si>
+  <si>
+    <t>Architecture</t>
+  </si>
+  <si>
+    <t>Tách code UI thành modules</t>
+  </si>
+  <si>
+    <t>Dễ maintain</t>
+  </si>
+  <si>
+    <t>Tránh file &gt;500 dòng</t>
+  </si>
+  <si>
+    <t>POD-001</t>
+  </si>
+  <si>
+    <t>Podcast Learning</t>
+  </si>
+  <si>
+    <t>Hiển thị danh sách podcast show từ DB sau login</t>
+  </si>
+  <si>
+    <t>Giảm thao tác nhập link</t>
+  </si>
+  <si>
+    <t>DB Shows</t>
+  </si>
+  <si>
+    <t>Mặc định hiển thị sẵn</t>
+  </si>
+  <si>
+    <t>POD-002</t>
+  </si>
+  <si>
+    <t>Cho phép nhập RSS/URL nếu show chưa có</t>
+  </si>
+  <si>
+    <t>Mở rộng nội dung</t>
+  </si>
+  <si>
+    <t>Fallback</t>
+  </si>
+  <si>
+    <t>POD-003</t>
+  </si>
+  <si>
+    <t>Hiển thị danh sách episodes của show</t>
+  </si>
+  <si>
+    <t>Chọn bài học dễ dàng</t>
+  </si>
+  <si>
+    <t>Episode browser</t>
+  </si>
+  <si>
+    <t>POD-004</t>
+  </si>
+  <si>
+    <t>Embedded audio player</t>
+  </si>
+  <si>
+    <t>Trải nghiệm học</t>
+  </si>
+  <si>
+    <t>Core feature</t>
+  </si>
+  <si>
+    <t>POD-005</t>
+  </si>
+  <si>
+    <t>Transcript đồng bộ audio</t>
+  </si>
+  <si>
+    <t>Tăng khả năng nghe hiểu</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Sentence level sync</t>
+  </si>
+  <si>
+    <t>POD-006</t>
+  </si>
+  <si>
+    <t>Highlight transcript theo audio time</t>
+  </si>
+  <si>
+    <t>Theo dõi dễ dàng</t>
+  </si>
+  <si>
+    <t>Karaoke style</t>
+  </si>
+  <si>
+    <t>POD-007</t>
+  </si>
+  <si>
+    <t>Click transcript để jump audio</t>
+  </si>
+  <si>
+    <t>Học nhanh</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>PMF</t>
+  </si>
+  <si>
+    <t>Optional</t>
+  </si>
+  <si>
+    <t>ANA-001</t>
+  </si>
+  <si>
+    <t>Analytics</t>
+  </si>
+  <si>
+    <t>Lưu lịch sử học</t>
+  </si>
+  <si>
+    <t>Tracking tiến độ</t>
+  </si>
+  <si>
+    <t>User Profile</t>
+  </si>
+  <si>
+    <t>ANA-002</t>
+  </si>
+  <si>
+    <t>Dashboard học tập</t>
+  </si>
+  <si>
+    <t>Theo dõi kết quả</t>
+  </si>
+  <si>
+    <t>ANA-003</t>
+  </si>
+  <si>
+    <t>Learning Progress</t>
+  </si>
+  <si>
+    <t>Tạo động lực</t>
+  </si>
+  <si>
+    <t>ANA-004</t>
+  </si>
+  <si>
+    <t>Streak Tracking</t>
+  </si>
+  <si>
+    <t>Retention</t>
+  </si>
+  <si>
+    <t>ANA-005</t>
+  </si>
+  <si>
+    <t>Daily Challenge</t>
+  </si>
+  <si>
+    <t>Engagement</t>
+  </si>
+  <si>
+    <t>ANA-006</t>
+  </si>
+  <si>
+    <t>Leaderboard</t>
+  </si>
+  <si>
+    <t>Gamification</t>
+  </si>
+  <si>
+    <t>AI-001</t>
+  </si>
+  <si>
+    <t>AI Coach</t>
+  </si>
+  <si>
+    <t>AI Pronunciation Scoring</t>
+  </si>
+  <si>
+    <t>Speaking improvement</t>
+  </si>
+  <si>
+    <t>Speaking Engine</t>
+  </si>
+  <si>
+    <t>AI-002</t>
+  </si>
+  <si>
+    <t>AI Conversation</t>
+  </si>
+  <si>
+    <t>Speaking practice</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>XL</t>
+  </si>
+  <si>
+    <t>AI Infra</t>
+  </si>
+  <si>
+    <t>AI-003</t>
+  </si>
+  <si>
+    <t>Roleplay Mode</t>
+  </si>
+  <si>
+    <t>Interactive learning</t>
+  </si>
+  <si>
+    <t>AI-004</t>
+  </si>
+  <si>
+    <t>Writing Correction</t>
+  </si>
+  <si>
+    <t>Writing skill</t>
+  </si>
+  <si>
+    <t>AI-005</t>
+  </si>
+  <si>
+    <t>Reading Quiz</t>
+  </si>
+  <si>
+    <t>Reading skill</t>
+  </si>
+  <si>
+    <t>Content Engine</t>
+  </si>
+  <si>
+    <t>MON-001</t>
+  </si>
+  <si>
+    <t>Monetization</t>
+  </si>
+  <si>
+    <t>Premium AI Speaking</t>
+  </si>
+  <si>
+    <t>Revenue</t>
+  </si>
+  <si>
+    <t>P3</t>
+  </si>
+  <si>
+    <t>MON-002</t>
+  </si>
+  <si>
+    <t>Premium Writing Feedback</t>
+  </si>
+  <si>
+    <t>MON-003</t>
+  </si>
+  <si>
+    <t>Advanced Analytics</t>
+  </si>
+  <si>
+    <t>MON-004</t>
+  </si>
+  <si>
+    <t>Podcast System</t>
+  </si>
+  <si>
+    <t>IELTS-001</t>
+  </si>
+  <si>
+    <t>IELTS Listening</t>
+  </si>
+  <si>
+    <t>Exam prep</t>
+  </si>
+  <si>
+    <t>P4</t>
+  </si>
+  <si>
+    <t>Existing Listening</t>
+  </si>
+  <si>
+    <t>IELTS-002</t>
+  </si>
+  <si>
+    <t>IELTS Reading</t>
+  </si>
+  <si>
+    <t>Quiz Engine</t>
+  </si>
+  <si>
+    <t>IELTS-003</t>
+  </si>
+  <si>
+    <t>IELTS Writing</t>
+  </si>
+  <si>
+    <t>AI Writing</t>
+  </si>
+  <si>
+    <t>IELTS-004</t>
+  </si>
+  <si>
+    <t>IELTS Speaking</t>
+  </si>
+  <si>
+    <t>AI Speaking</t>
+  </si>
+  <si>
+    <t>IELTS-005</t>
+  </si>
+  <si>
+    <t>AI Examiner</t>
+  </si>
+  <si>
+    <t>Simulation</t>
+  </si>
+  <si>
+    <t>IELTS Modules</t>
+  </si>
+  <si>
+    <t>B2B-001</t>
+  </si>
+  <si>
+    <t>B2B Education</t>
+  </si>
+  <si>
+    <t>Teacher management</t>
+  </si>
+  <si>
+    <t>P5</t>
+  </si>
+  <si>
+    <t>B2B-002</t>
+  </si>
+  <si>
+    <t>User Management</t>
+  </si>
+  <si>
+    <t>B2B-003</t>
+  </si>
+  <si>
+    <t>Báo cáo tiến độ học viên</t>
+  </si>
+  <si>
+    <t>Teacher insights</t>
+  </si>
+  <si>
+    <t>HSK-001</t>
+  </si>
+  <si>
+    <t>Listening</t>
+  </si>
+  <si>
+    <t>Chinese learning</t>
+  </si>
+  <si>
+    <t>P6</t>
+  </si>
+  <si>
+    <t>English Framework</t>
+  </si>
+  <si>
+    <t>HSK-002</t>
+  </si>
+  <si>
+    <t>Speaking</t>
+  </si>
+  <si>
+    <t>HSK-003</t>
+  </si>
+  <si>
+    <t>Reading</t>
+  </si>
+  <si>
+    <t>HSK-004</t>
+  </si>
+  <si>
+    <t>Writing</t>
+  </si>
+  <si>
+    <t>EDU-001</t>
+  </si>
+  <si>
+    <t>K12 Education</t>
+  </si>
+  <si>
+    <t>Toán lớp 8</t>
+  </si>
+  <si>
+    <t>K12 market</t>
+  </si>
+  <si>
+    <t>P8</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+  <si>
+    <t>Learning Platform</t>
+  </si>
+  <si>
+    <t>EDU-002</t>
+  </si>
+  <si>
+    <t>KHTN lớp 8</t>
+  </si>
+  <si>
+    <t>EDU-003</t>
+  </si>
+  <si>
+    <t>Tiếng Anh SGK</t>
+  </si>
+  <si>
+    <t>EDU-004</t>
+  </si>
+  <si>
+    <t>AI Tutor</t>
+  </si>
+  <si>
+    <t>EDU-005</t>
+  </si>
+  <si>
+    <t>Quiz System</t>
+  </si>
+  <si>
+    <t>Assessment</t>
+  </si>
+  <si>
+    <t>New</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -684,6 +1512,14 @@
     <font>
       <b/>
       <sz val="13.5"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -716,7 +1552,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -766,6 +1602,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1932,7 +2771,1581 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:L50"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="41.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="36.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="31" x14ac:dyDescent="0.35">
+      <c r="A1" s="19" t="s">
+        <v>280</v>
+      </c>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B3" s="13" t="s">
+        <v>281</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="G3" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>287</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="K3" s="13" t="s">
+        <v>290</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B4" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>292</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>293</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>294</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="G4" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H4" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="I4" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J4" s="16" t="s">
+        <v>299</v>
+      </c>
+      <c r="K4" s="16" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B5" s="16" t="s">
+        <v>301</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>292</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="I5" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J5" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="K5" s="16" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B6" s="16" t="s">
+        <v>305</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>292</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>306</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>307</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H6" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="I6" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J6" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="K6" s="16" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B7" s="16" t="s">
+        <v>309</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>292</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>310</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>311</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>312</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="I7" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J7" s="16" t="s">
+        <v>299</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B8" s="16" t="s">
+        <v>314</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>292</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>315</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>316</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>312</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="I8" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J8" s="16" t="s">
+        <v>299</v>
+      </c>
+      <c r="K8" s="16" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B9" s="16" t="s">
+        <v>318</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>292</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>319</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>320</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H9" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="I9" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J9" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B10" s="16" t="s">
+        <v>322</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>292</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>323</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>324</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>312</v>
+      </c>
+      <c r="H10" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="I10" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J10" s="16" t="s">
+        <v>299</v>
+      </c>
+      <c r="K10" s="16" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B11" s="16" t="s">
+        <v>326</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>327</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>328</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>329</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="G11" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H11" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="I11" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J11" s="16" t="s">
+        <v>299</v>
+      </c>
+      <c r="K11" s="16" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B12" s="16" t="s">
+        <v>331</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>332</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>333</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>334</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="G12" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H12" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="I12" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J12" s="16" t="s">
+        <v>335</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B13" s="16" t="s">
+        <v>337</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>332</v>
+      </c>
+      <c r="D13" s="16" t="s">
+        <v>338</v>
+      </c>
+      <c r="E13" s="16" t="s">
+        <v>339</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="G13" s="16" t="s">
+        <v>312</v>
+      </c>
+      <c r="H13" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="I13" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J13" s="16" t="s">
+        <v>331</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B14" s="16" t="s">
+        <v>341</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>332</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>342</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>343</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="I14" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J14" s="16" t="s">
+        <v>331</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B15" s="16" t="s">
+        <v>345</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>332</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>346</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>347</v>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="G15" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H15" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="I15" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J15" s="16" t="s">
+        <v>341</v>
+      </c>
+      <c r="K15" s="16" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B16" s="16" t="s">
+        <v>349</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>332</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>350</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>351</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="G16" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="H16" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="I16" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J16" s="16" t="s">
+        <v>345</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B17" s="16" t="s">
+        <v>354</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>332</v>
+      </c>
+      <c r="D17" s="16" t="s">
+        <v>355</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>356</v>
+      </c>
+      <c r="F17" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="G17" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="H17" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="I17" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J17" s="16" t="s">
+        <v>349</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B18" s="16" t="s">
+        <v>358</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>332</v>
+      </c>
+      <c r="D18" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="E18" s="16" t="s">
+        <v>360</v>
+      </c>
+      <c r="F18" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="G18" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H18" s="16" t="s">
+        <v>362</v>
+      </c>
+      <c r="I18" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J18" s="16" t="s">
+        <v>354</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B19" s="16" t="s">
+        <v>364</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="D19" s="16" t="s">
+        <v>366</v>
+      </c>
+      <c r="E19" s="16" t="s">
+        <v>367</v>
+      </c>
+      <c r="F19" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="G19" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H19" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="I19" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J19" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="K19" s="16"/>
+    </row>
+    <row r="20" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B20" s="16" t="s">
+        <v>369</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="D20" s="16" t="s">
+        <v>370</v>
+      </c>
+      <c r="E20" s="16" t="s">
+        <v>371</v>
+      </c>
+      <c r="F20" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="G20" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H20" s="16" t="s">
+        <v>362</v>
+      </c>
+      <c r="I20" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J20" s="16" t="s">
+        <v>364</v>
+      </c>
+      <c r="K20" s="16"/>
+    </row>
+    <row r="21" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B21" s="16" t="s">
+        <v>372</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="D21" s="16" t="s">
+        <v>373</v>
+      </c>
+      <c r="E21" s="16" t="s">
+        <v>374</v>
+      </c>
+      <c r="F21" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="G21" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H21" s="16" t="s">
+        <v>362</v>
+      </c>
+      <c r="I21" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J21" s="16" t="s">
+        <v>369</v>
+      </c>
+      <c r="K21" s="16"/>
+    </row>
+    <row r="22" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B22" s="16" t="s">
+        <v>375</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="D22" s="16" t="s">
+        <v>376</v>
+      </c>
+      <c r="E22" s="16" t="s">
+        <v>377</v>
+      </c>
+      <c r="F22" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="G22" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H22" s="16" t="s">
+        <v>362</v>
+      </c>
+      <c r="I22" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J22" s="16" t="s">
+        <v>364</v>
+      </c>
+      <c r="K22" s="16"/>
+    </row>
+    <row r="23" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B23" s="16" t="s">
+        <v>378</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="D23" s="16" t="s">
+        <v>379</v>
+      </c>
+      <c r="E23" s="16" t="s">
+        <v>380</v>
+      </c>
+      <c r="F23" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="G23" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H23" s="16" t="s">
+        <v>362</v>
+      </c>
+      <c r="I23" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J23" s="16" t="s">
+        <v>375</v>
+      </c>
+      <c r="K23" s="16"/>
+    </row>
+    <row r="24" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B24" s="16" t="s">
+        <v>381</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="D24" s="16" t="s">
+        <v>382</v>
+      </c>
+      <c r="E24" s="16" t="s">
+        <v>383</v>
+      </c>
+      <c r="F24" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="G24" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H24" s="16" t="s">
+        <v>362</v>
+      </c>
+      <c r="I24" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J24" s="16" t="s">
+        <v>375</v>
+      </c>
+      <c r="K24" s="16"/>
+    </row>
+    <row r="25" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B25" s="16" t="s">
+        <v>384</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="D25" s="16" t="s">
+        <v>386</v>
+      </c>
+      <c r="E25" s="16" t="s">
+        <v>387</v>
+      </c>
+      <c r="F25" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="G25" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="H25" s="16" t="s">
+        <v>362</v>
+      </c>
+      <c r="I25" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J25" s="16" t="s">
+        <v>388</v>
+      </c>
+      <c r="K25" s="16"/>
+    </row>
+    <row r="26" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B26" s="16" t="s">
+        <v>389</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="D26" s="16" t="s">
+        <v>390</v>
+      </c>
+      <c r="E26" s="16" t="s">
+        <v>391</v>
+      </c>
+      <c r="F26" s="16" t="s">
+        <v>392</v>
+      </c>
+      <c r="G26" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="H26" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="I26" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J26" s="16" t="s">
+        <v>394</v>
+      </c>
+      <c r="K26" s="16"/>
+    </row>
+    <row r="27" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B27" s="16" t="s">
+        <v>395</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="D27" s="16" t="s">
+        <v>396</v>
+      </c>
+      <c r="E27" s="16" t="s">
+        <v>397</v>
+      </c>
+      <c r="F27" s="16" t="s">
+        <v>392</v>
+      </c>
+      <c r="G27" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="H27" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="I27" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J27" s="16" t="s">
+        <v>389</v>
+      </c>
+      <c r="K27" s="16"/>
+    </row>
+    <row r="28" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B28" s="16" t="s">
+        <v>398</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>399</v>
+      </c>
+      <c r="E28" s="16" t="s">
+        <v>400</v>
+      </c>
+      <c r="F28" s="16" t="s">
+        <v>392</v>
+      </c>
+      <c r="G28" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="H28" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="I28" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J28" s="16" t="s">
+        <v>394</v>
+      </c>
+      <c r="K28" s="16"/>
+    </row>
+    <row r="29" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B29" s="16" t="s">
+        <v>401</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="D29" s="16" t="s">
+        <v>402</v>
+      </c>
+      <c r="E29" s="16" t="s">
+        <v>403</v>
+      </c>
+      <c r="F29" s="16" t="s">
+        <v>392</v>
+      </c>
+      <c r="G29" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H29" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="I29" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J29" s="16" t="s">
+        <v>404</v>
+      </c>
+      <c r="K29" s="16"/>
+    </row>
+    <row r="30" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B30" s="16" t="s">
+        <v>405</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>406</v>
+      </c>
+      <c r="D30" s="16" t="s">
+        <v>407</v>
+      </c>
+      <c r="E30" s="16" t="s">
+        <v>408</v>
+      </c>
+      <c r="F30" s="16" t="s">
+        <v>409</v>
+      </c>
+      <c r="G30" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H30" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="I30" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J30" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="K30" s="16"/>
+    </row>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B31" s="16" t="s">
+        <v>410</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>406</v>
+      </c>
+      <c r="D31" s="16" t="s">
+        <v>411</v>
+      </c>
+      <c r="E31" s="16" t="s">
+        <v>408</v>
+      </c>
+      <c r="F31" s="16" t="s">
+        <v>409</v>
+      </c>
+      <c r="G31" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H31" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="I31" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J31" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="K31" s="16"/>
+    </row>
+    <row r="32" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B32" s="16" t="s">
+        <v>412</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>406</v>
+      </c>
+      <c r="D32" s="16" t="s">
+        <v>413</v>
+      </c>
+      <c r="E32" s="16" t="s">
+        <v>408</v>
+      </c>
+      <c r="F32" s="16" t="s">
+        <v>409</v>
+      </c>
+      <c r="G32" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H32" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="I32" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J32" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="K32" s="16"/>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B33" s="16" t="s">
+        <v>414</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>406</v>
+      </c>
+      <c r="D33" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E33" s="16" t="s">
+        <v>408</v>
+      </c>
+      <c r="F33" s="16" t="s">
+        <v>409</v>
+      </c>
+      <c r="G33" s="16" t="s">
+        <v>312</v>
+      </c>
+      <c r="H33" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="I33" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J33" s="16" t="s">
+        <v>415</v>
+      </c>
+      <c r="K33" s="16"/>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B34" s="16" t="s">
+        <v>416</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="D34" s="16" t="s">
+        <v>417</v>
+      </c>
+      <c r="E34" s="16" t="s">
+        <v>418</v>
+      </c>
+      <c r="F34" s="16" t="s">
+        <v>419</v>
+      </c>
+      <c r="G34" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="H34" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="I34" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J34" s="16" t="s">
+        <v>420</v>
+      </c>
+      <c r="K34" s="16"/>
+      <c r="L34" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B35" s="16" t="s">
+        <v>421</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="D35" s="16" t="s">
+        <v>422</v>
+      </c>
+      <c r="E35" s="16" t="s">
+        <v>418</v>
+      </c>
+      <c r="F35" s="16" t="s">
+        <v>419</v>
+      </c>
+      <c r="G35" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="H35" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="I35" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J35" s="16" t="s">
+        <v>423</v>
+      </c>
+      <c r="K35" s="16"/>
+      <c r="L35" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B36" s="16" t="s">
+        <v>424</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="D36" s="16" t="s">
+        <v>425</v>
+      </c>
+      <c r="E36" s="16" t="s">
+        <v>418</v>
+      </c>
+      <c r="F36" s="16" t="s">
+        <v>419</v>
+      </c>
+      <c r="G36" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="H36" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="I36" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J36" s="16" t="s">
+        <v>426</v>
+      </c>
+      <c r="K36" s="16"/>
+      <c r="L36" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B37" s="16" t="s">
+        <v>427</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="D37" s="16" t="s">
+        <v>428</v>
+      </c>
+      <c r="E37" s="16" t="s">
+        <v>418</v>
+      </c>
+      <c r="F37" s="16" t="s">
+        <v>419</v>
+      </c>
+      <c r="G37" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="H37" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="I37" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J37" s="16" t="s">
+        <v>429</v>
+      </c>
+      <c r="K37" s="16"/>
+      <c r="L37" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B38" s="16" t="s">
+        <v>430</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="D38" s="16" t="s">
+        <v>431</v>
+      </c>
+      <c r="E38" s="16" t="s">
+        <v>432</v>
+      </c>
+      <c r="F38" s="16" t="s">
+        <v>419</v>
+      </c>
+      <c r="G38" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="H38" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="I38" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J38" s="16" t="s">
+        <v>433</v>
+      </c>
+      <c r="K38" s="16"/>
+      <c r="L38" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B39" s="16" t="s">
+        <v>434</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>435</v>
+      </c>
+      <c r="D39" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E39" s="16" t="s">
+        <v>436</v>
+      </c>
+      <c r="F39" s="16" t="s">
+        <v>437</v>
+      </c>
+      <c r="G39" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="H39" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="I39" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J39" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="K39" s="16"/>
+      <c r="L39" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B40" s="16" t="s">
+        <v>438</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>435</v>
+      </c>
+      <c r="D40" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="E40" s="16" t="s">
+        <v>436</v>
+      </c>
+      <c r="F40" s="16" t="s">
+        <v>437</v>
+      </c>
+      <c r="G40" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="H40" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="I40" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J40" s="16" t="s">
+        <v>439</v>
+      </c>
+      <c r="K40" s="16"/>
+      <c r="L40" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B41" s="16" t="s">
+        <v>440</v>
+      </c>
+      <c r="C41" s="16" t="s">
+        <v>435</v>
+      </c>
+      <c r="D41" s="16" t="s">
+        <v>441</v>
+      </c>
+      <c r="E41" s="16" t="s">
+        <v>442</v>
+      </c>
+      <c r="F41" s="16" t="s">
+        <v>437</v>
+      </c>
+      <c r="G41" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="H41" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="I41" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J41" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="K41" s="16"/>
+      <c r="L41" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B42" s="16" t="s">
+        <v>443</v>
+      </c>
+      <c r="C42" s="16" t="s">
+        <v>198</v>
+      </c>
+      <c r="D42" s="16" t="s">
+        <v>444</v>
+      </c>
+      <c r="E42" s="16" t="s">
+        <v>445</v>
+      </c>
+      <c r="F42" s="16" t="s">
+        <v>446</v>
+      </c>
+      <c r="G42" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H42" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="I42" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J42" s="16" t="s">
+        <v>447</v>
+      </c>
+      <c r="K42" s="16"/>
+      <c r="L42" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B43" s="16" t="s">
+        <v>448</v>
+      </c>
+      <c r="C43" s="16" t="s">
+        <v>198</v>
+      </c>
+      <c r="D43" s="16" t="s">
+        <v>449</v>
+      </c>
+      <c r="E43" s="16" t="s">
+        <v>445</v>
+      </c>
+      <c r="F43" s="16" t="s">
+        <v>446</v>
+      </c>
+      <c r="G43" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H43" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="I43" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J43" s="16" t="s">
+        <v>447</v>
+      </c>
+      <c r="K43" s="16"/>
+      <c r="L43" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B44" s="16" t="s">
+        <v>450</v>
+      </c>
+      <c r="C44" s="16" t="s">
+        <v>198</v>
+      </c>
+      <c r="D44" s="16" t="s">
+        <v>451</v>
+      </c>
+      <c r="E44" s="16" t="s">
+        <v>445</v>
+      </c>
+      <c r="F44" s="16" t="s">
+        <v>446</v>
+      </c>
+      <c r="G44" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H44" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="I44" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J44" s="16" t="s">
+        <v>447</v>
+      </c>
+      <c r="K44" s="16"/>
+      <c r="L44" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B45" s="16" t="s">
+        <v>452</v>
+      </c>
+      <c r="C45" s="16" t="s">
+        <v>198</v>
+      </c>
+      <c r="D45" s="16" t="s">
+        <v>453</v>
+      </c>
+      <c r="E45" s="16" t="s">
+        <v>445</v>
+      </c>
+      <c r="F45" s="16" t="s">
+        <v>446</v>
+      </c>
+      <c r="G45" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="H45" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="I45" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J45" s="16" t="s">
+        <v>447</v>
+      </c>
+      <c r="K45" s="16"/>
+      <c r="L45" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B46" s="16" t="s">
+        <v>454</v>
+      </c>
+      <c r="C46" s="16" t="s">
+        <v>455</v>
+      </c>
+      <c r="D46" s="16" t="s">
+        <v>456</v>
+      </c>
+      <c r="E46" s="16" t="s">
+        <v>457</v>
+      </c>
+      <c r="F46" s="16" t="s">
+        <v>458</v>
+      </c>
+      <c r="G46" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="H46" s="16" t="s">
+        <v>459</v>
+      </c>
+      <c r="I46" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J46" s="16" t="s">
+        <v>460</v>
+      </c>
+      <c r="K46" s="16"/>
+      <c r="L46" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="47" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B47" s="16" t="s">
+        <v>461</v>
+      </c>
+      <c r="C47" s="16" t="s">
+        <v>455</v>
+      </c>
+      <c r="D47" s="16" t="s">
+        <v>462</v>
+      </c>
+      <c r="E47" s="16" t="s">
+        <v>457</v>
+      </c>
+      <c r="F47" s="16" t="s">
+        <v>458</v>
+      </c>
+      <c r="G47" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="H47" s="16" t="s">
+        <v>459</v>
+      </c>
+      <c r="I47" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J47" s="16" t="s">
+        <v>460</v>
+      </c>
+      <c r="K47" s="16"/>
+      <c r="L47" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B48" s="16" t="s">
+        <v>463</v>
+      </c>
+      <c r="C48" s="16" t="s">
+        <v>455</v>
+      </c>
+      <c r="D48" s="16" t="s">
+        <v>464</v>
+      </c>
+      <c r="E48" s="16" t="s">
+        <v>457</v>
+      </c>
+      <c r="F48" s="16" t="s">
+        <v>458</v>
+      </c>
+      <c r="G48" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="H48" s="16" t="s">
+        <v>459</v>
+      </c>
+      <c r="I48" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J48" s="16" t="s">
+        <v>460</v>
+      </c>
+      <c r="K48" s="16"/>
+      <c r="L48" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="49" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B49" s="16" t="s">
+        <v>465</v>
+      </c>
+      <c r="C49" s="16" t="s">
+        <v>455</v>
+      </c>
+      <c r="D49" s="16" t="s">
+        <v>466</v>
+      </c>
+      <c r="E49" s="16" t="s">
+        <v>457</v>
+      </c>
+      <c r="F49" s="16" t="s">
+        <v>458</v>
+      </c>
+      <c r="G49" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="H49" s="16" t="s">
+        <v>459</v>
+      </c>
+      <c r="I49" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J49" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="K49" s="16"/>
+      <c r="L49" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="50" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B50" s="16" t="s">
+        <v>467</v>
+      </c>
+      <c r="C50" s="16" t="s">
+        <v>455</v>
+      </c>
+      <c r="D50" s="16" t="s">
+        <v>468</v>
+      </c>
+      <c r="E50" s="16" t="s">
+        <v>469</v>
+      </c>
+      <c r="F50" s="16" t="s">
+        <v>458</v>
+      </c>
+      <c r="G50" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="H50" s="16" t="s">
+        <v>459</v>
+      </c>
+      <c r="I50" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="J50" s="16" t="s">
+        <v>460</v>
+      </c>
+      <c r="K50" s="16"/>
+      <c r="L50" s="16" t="s">
+        <v>470</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C126"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.1796875" style="14" bestFit="1" customWidth="1"/>
@@ -1985,12 +4398,654 @@
         <v>151</v>
       </c>
     </row>
+    <row r="6" spans="1:3" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="B6" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="C6"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B7"/>
+      <c r="C7"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>209</v>
+      </c>
+      <c r="C8"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B9" s="6"/>
+      <c r="C9"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B10" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="C10"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B11" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="C11"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B12"/>
+      <c r="C12"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>212</v>
+      </c>
+      <c r="C13"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B14"/>
+      <c r="C14"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B15" t="s">
+        <v>213</v>
+      </c>
+      <c r="C15"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B16"/>
+      <c r="C16"/>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B17" t="s">
+        <v>209</v>
+      </c>
+      <c r="C17"/>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B18" s="6"/>
+      <c r="C18"/>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B19" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="C19"/>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B20" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="C20"/>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B21"/>
+      <c r="C21"/>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B22" t="s">
+        <v>216</v>
+      </c>
+      <c r="C22"/>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B23"/>
+      <c r="C23"/>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B24"/>
+      <c r="C24"/>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B25"/>
+      <c r="C25"/>
+    </row>
+    <row r="26" spans="2:3" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="B26" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="C26"/>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B27"/>
+      <c r="C27"/>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B28" t="s">
+        <v>218</v>
+      </c>
+      <c r="C28"/>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B29"/>
+      <c r="C29"/>
+    </row>
+    <row r="30" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B30" t="s">
+        <v>209</v>
+      </c>
+      <c r="C30"/>
+    </row>
+    <row r="31" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B31"/>
+      <c r="C31"/>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B32" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B33" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="C33" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B34" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="C34" s="3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B35" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="C35" s="3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B36" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="C36" s="3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B37"/>
+      <c r="C37"/>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B38" t="s">
+        <v>225</v>
+      </c>
+      <c r="C38"/>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B39"/>
+      <c r="C39"/>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B40" t="s">
+        <v>226</v>
+      </c>
+      <c r="C40"/>
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B41" s="6"/>
+      <c r="C41"/>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B42" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="C42"/>
+    </row>
+    <row r="43" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B43" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="C43"/>
+    </row>
+    <row r="44" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B44" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="C44"/>
+    </row>
+    <row r="45" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B45"/>
+      <c r="C45"/>
+    </row>
+    <row r="46" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B46"/>
+      <c r="C46"/>
+    </row>
+    <row r="47" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B47"/>
+      <c r="C47"/>
+    </row>
+    <row r="48" spans="2:3" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="B48" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="C48"/>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B49"/>
+      <c r="C49"/>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B50" t="s">
+        <v>231</v>
+      </c>
+      <c r="C50"/>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B51"/>
+      <c r="C51"/>
+    </row>
+    <row r="52" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B52" t="s">
+        <v>232</v>
+      </c>
+      <c r="C52"/>
+    </row>
+    <row r="53" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B53"/>
+      <c r="C53"/>
+    </row>
+    <row r="54" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B54" t="s">
+        <v>233</v>
+      </c>
+      <c r="C54"/>
+    </row>
+    <row r="55" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B55" s="6"/>
+      <c r="C55"/>
+    </row>
+    <row r="56" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B56" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="C56"/>
+    </row>
+    <row r="57" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B57"/>
+      <c r="C57"/>
+    </row>
+    <row r="58" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B58" t="s">
+        <v>235</v>
+      </c>
+      <c r="C58"/>
+    </row>
+    <row r="59" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B59" s="6"/>
+      <c r="C59"/>
+    </row>
+    <row r="60" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B60" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="C60"/>
+    </row>
+    <row r="61" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B61"/>
+      <c r="C61"/>
+    </row>
+    <row r="62" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B62" t="s">
+        <v>237</v>
+      </c>
+      <c r="C62"/>
+    </row>
+    <row r="63" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B63"/>
+      <c r="C63"/>
+    </row>
+    <row r="64" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B64" t="s">
+        <v>238</v>
+      </c>
+      <c r="C64"/>
+    </row>
+    <row r="65" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B65"/>
+      <c r="C65"/>
+    </row>
+    <row r="66" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B66" t="s">
+        <v>239</v>
+      </c>
+      <c r="C66"/>
+    </row>
+    <row r="67" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B67"/>
+      <c r="C67"/>
+    </row>
+    <row r="68" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B68"/>
+      <c r="C68"/>
+    </row>
+    <row r="69" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B69"/>
+      <c r="C69"/>
+    </row>
+    <row r="70" spans="2:3" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="B70" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="C70"/>
+    </row>
+    <row r="71" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B71"/>
+      <c r="C71"/>
+    </row>
+    <row r="72" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B72" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="73" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B73" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="74" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B74" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="75" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B75" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="76" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B76" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="77" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B77" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="78" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B78"/>
+      <c r="C78"/>
+    </row>
+    <row r="79" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B79" t="s">
+        <v>253</v>
+      </c>
+      <c r="C79"/>
+    </row>
+    <row r="80" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B80" s="6"/>
+      <c r="C80"/>
+    </row>
+    <row r="81" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B81" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="C81"/>
+    </row>
+    <row r="82" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B82" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="C82"/>
+    </row>
+    <row r="83" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B83"/>
+      <c r="C83"/>
+    </row>
+    <row r="84" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B84"/>
+      <c r="C84"/>
+    </row>
+    <row r="85" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B85"/>
+      <c r="C85"/>
+    </row>
+    <row r="86" spans="2:3" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="B86" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="C86"/>
+    </row>
+    <row r="87" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B87"/>
+      <c r="C87"/>
+    </row>
+    <row r="88" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B88" t="s">
+        <v>257</v>
+      </c>
+      <c r="C88"/>
+    </row>
+    <row r="89" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B89" s="6"/>
+      <c r="C89"/>
+    </row>
+    <row r="90" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B90" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="C90"/>
+    </row>
+    <row r="91" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B91" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="C91"/>
+    </row>
+    <row r="92" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B92" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C92"/>
+    </row>
+    <row r="93" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B93"/>
+      <c r="C93"/>
+    </row>
+    <row r="94" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B94" t="s">
+        <v>260</v>
+      </c>
+      <c r="C94"/>
+    </row>
+    <row r="95" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B95"/>
+      <c r="C95"/>
+    </row>
+    <row r="96" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B96" t="s">
+        <v>261</v>
+      </c>
+      <c r="C96"/>
+    </row>
+    <row r="97" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B97" s="6"/>
+      <c r="C97"/>
+    </row>
+    <row r="98" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B98" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="C98"/>
+    </row>
+    <row r="99" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B99" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="C99"/>
+    </row>
+    <row r="100" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B100" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="C100"/>
+    </row>
+    <row r="101" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B101"/>
+      <c r="C101"/>
+    </row>
+    <row r="102" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B102" t="s">
+        <v>265</v>
+      </c>
+      <c r="C102"/>
+    </row>
+    <row r="103" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B103"/>
+      <c r="C103"/>
+    </row>
+    <row r="104" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B104"/>
+      <c r="C104"/>
+    </row>
+    <row r="105" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B105"/>
+      <c r="C105"/>
+    </row>
+    <row r="106" spans="2:3" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="B106" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="C106"/>
+    </row>
+    <row r="107" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B107"/>
+      <c r="C107"/>
+    </row>
+    <row r="108" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B108" t="s">
+        <v>267</v>
+      </c>
+      <c r="C108"/>
+    </row>
+    <row r="109" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B109"/>
+      <c r="C109"/>
+    </row>
+    <row r="110" spans="2:3" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="B110" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="C110"/>
+    </row>
+    <row r="111" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B111"/>
+      <c r="C111"/>
+    </row>
+    <row r="112" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B112" t="s">
+        <v>269</v>
+      </c>
+      <c r="C112"/>
+    </row>
+    <row r="113" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B113" s="6"/>
+      <c r="C113"/>
+    </row>
+    <row r="114" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B114" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="C114"/>
+    </row>
+    <row r="115" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B115" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C115"/>
+    </row>
+    <row r="116" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B116" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="C116"/>
+    </row>
+    <row r="117" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B117"/>
+      <c r="C117"/>
+    </row>
+    <row r="118" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B118" t="s">
+        <v>273</v>
+      </c>
+      <c r="C118"/>
+    </row>
+    <row r="119" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B119" s="6"/>
+      <c r="C119"/>
+    </row>
+    <row r="120" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B120" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="C120"/>
+    </row>
+    <row r="121" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B121" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="C121"/>
+    </row>
+    <row r="122" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B122" s="9" t="s">
+        <v>276</v>
+      </c>
+      <c r="C122"/>
+    </row>
+    <row r="123" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B123" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="C123"/>
+    </row>
+    <row r="124" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B124" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="C124"/>
+    </row>
+    <row r="125" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B125"/>
+      <c r="C125"/>
+    </row>
+    <row r="126" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B126" t="s">
+        <v>279</v>
+      </c>
+      <c r="C126"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>